<commit_message>
派 D15 (WiFi 端 12-bit 色深) / D16 (16 bit DDR 极限); 保存夜间安排
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-13.xlsx
+++ b/docs/progress/显性目的进度_2026-10-13.xlsx
@@ -12107,7 +12107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12151,7 +12151,7 @@
         <v>46307</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>5</v>
@@ -12165,7 +12165,7 @@
         <v>46308</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>7</v>
@@ -12179,7 +12179,7 @@
         <v>46309</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>8</v>
@@ -12191,7 +12191,7 @@
         <v>46310</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>10</v>
@@ -12203,7 +12203,7 @@
         <v>46311</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>15</v>
@@ -12215,10 +12215,10 @@
         <v>46312</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9" s="3" t="n"/>
     </row>
@@ -12227,10 +12227,10 @@
         <v>46313</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3" t="n"/>
     </row>
@@ -12239,10 +12239,10 @@
         <v>46314</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D11" s="3" t="n"/>
     </row>
@@ -12251,10 +12251,10 @@
         <v>46315</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D12" s="3" t="n"/>
     </row>
@@ -12263,10 +12263,10 @@
         <v>46316</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D13" s="3" t="n"/>
     </row>
@@ -12275,10 +12275,10 @@
         <v>46317</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D14" s="3" t="n"/>
     </row>
@@ -12287,10 +12287,10 @@
         <v>46318</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D15" s="3" t="n"/>
     </row>
@@ -12299,10 +12299,10 @@
         <v>46319</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D16" s="3" t="n"/>
     </row>
@@ -13130,6 +13130,78 @@
       <c r="H45" s="6" t="inlineStr">
         <is>
           <t>task/d14-content</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>WiFi 端 12-bit 色深通路 (像素位宽 16/32 可配)</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>task/d15-color</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>16 bit DDR 做到极限 (A 线: 慢读定位/分端口/预取缓冲/兜底)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>7;2</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>task/d16-ddr</t>
         </is>
       </c>
     </row>

</xml_diff>